<commit_message>
tools enhanced version 4.0
</commit_message>
<xml_diff>
--- a/data/input/test_addresses.xlsx
+++ b/data/input/test_addresses.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahulgupta/Documents/Coding/structured_address_ai_poc/data/samples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahulgupta/Documents/Coding/structured_address_ai_poc/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CB6B26-4005-F646-8555-E17A3D2B643C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7507FBD6-06A7-A944-8A0B-5AC5A21555A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{6F07F338-D208-7A41-832C-031358500E4C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>Addr_1</t>
   </si>
@@ -186,6 +186,36 @@
   </si>
   <si>
     <t>ES</t>
+  </si>
+  <si>
+    <t>Villa E5, Malee Beach, 541/2 Moo 2</t>
+  </si>
+  <si>
+    <t>Long Beach Pra-Ae Beach</t>
+  </si>
+  <si>
+    <t>81150 Krabi, Thailand</t>
+  </si>
+  <si>
+    <t>Plot 16-B</t>
+  </si>
+  <si>
+    <t>Punjab Small Industries Estate</t>
+  </si>
+  <si>
+    <t>Jhang Bahtra Road, Taxila</t>
+  </si>
+  <si>
+    <t>PK</t>
+  </si>
+  <si>
+    <t>Parc d'activities du plateau de sign</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>Italy</t>
   </si>
 </sst>
 </file>
@@ -557,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DFABB4-F73B-044C-B027-E58C429E5B49}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -753,6 +783,47 @@
         <v>49</v>
       </c>
     </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>